<commit_message>
Add Visual Studio solution and competitor comparison on Plans sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnFkPErZAiR8ShyLR6FSvf
</commit_message>
<xml_diff>
--- a/excel/SmartTrader_ERP_C.xlsx
+++ b/excel/SmartTrader_ERP_C.xlsx
@@ -238,7 +238,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -371,6 +371,12 @@
         <bgColor rgb="005E35B1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -411,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -655,6 +661,24 @@
     </xf>
     <xf numFmtId="170" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3397,14 +3421,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3745,6 +3769,130 @@
       <c r="B28" s="70" t="inlineStr">
         <is>
           <t xml:space="preserve">     entered beyond the Free limit were kept and are counted the moment Pro is active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="123" t="inlineStr">
+        <is>
+          <t>HOW PRO COMPARES (yearly price, Oct 2026 listings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="126" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C31" s="127" t="inlineStr">
+        <is>
+          <t>Price / year</t>
+        </is>
+      </c>
+      <c r="D31" s="127" t="inlineStr">
+        <is>
+          <t>Per month</t>
+        </is>
+      </c>
+      <c r="E31" s="126" t="inlineStr">
+        <is>
+          <t>Works offline, your data stays in your file</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="128" t="inlineStr">
+        <is>
+          <t>SmartTrader Pro (this file)</t>
+        </is>
+      </c>
+      <c r="C32" s="129" t="inlineStr">
+        <is>
+          <t>Rs 1,299</t>
+        </is>
+      </c>
+      <c r="D32" s="129" t="inlineStr">
+        <is>
+          <t>Rs 108</t>
+        </is>
+      </c>
+      <c r="E32" s="128" t="inlineStr">
+        <is>
+          <t>Yes - plain Excel, no login</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="130" t="inlineStr">
+        <is>
+          <t>myBillBook Plus / Pro</t>
+        </is>
+      </c>
+      <c r="C33" s="131" t="inlineStr">
+        <is>
+          <t>Rs 3,490 - 3,990</t>
+        </is>
+      </c>
+      <c r="D33" s="131" t="inlineStr">
+        <is>
+          <t>Rs 291 - 333</t>
+        </is>
+      </c>
+      <c r="E33" s="130" t="inlineStr">
+        <is>
+          <t>Cloud account</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="130" t="inlineStr">
+        <is>
+          <t>Vyapar Desktop</t>
+        </is>
+      </c>
+      <c r="C34" s="131" t="inlineStr">
+        <is>
+          <t>Rs 3,399 - 4,099</t>
+        </is>
+      </c>
+      <c r="D34" s="131" t="inlineStr">
+        <is>
+          <t>Rs 283 - 342</t>
+        </is>
+      </c>
+      <c r="E34" s="130" t="inlineStr">
+        <is>
+          <t>Desktop app</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="130" t="inlineStr">
+        <is>
+          <t>TallyPrime Silver (rental)</t>
+        </is>
+      </c>
+      <c r="C35" s="131" t="inlineStr">
+        <is>
+          <t>Rs 8,100</t>
+        </is>
+      </c>
+      <c r="D35" s="131" t="inlineStr">
+        <is>
+          <t>Rs 675</t>
+        </is>
+      </c>
+      <c r="E35" s="130" t="inlineStr">
+        <is>
+          <t>Desktop app</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Competitor prices are public listings and change often; they include cloud/mobile features this file does not.</t>
         </is>
       </c>
     </row>
@@ -3795,7 +3943,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="126" t="inlineStr">
+      <c r="B4" s="132" t="inlineStr">
         <is>
           <t>DAILY FLOW: PROCURE → STOCK → SELL → DELIVER → COLLECT</t>
         </is>
@@ -3803,103 +3951,103 @@
       <c r="C4" s="57" t="n"/>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="127" t="inlineStr">
+      <c r="B5" s="133" t="inlineStr">
         <is>
           <t>1. Set up once</t>
         </is>
       </c>
-      <c r="C5" s="128" t="inlineStr">
+      <c r="C5" s="134" t="inlineStr">
         <is>
           <t>Settings: company, GSTIN, home state, FY start, opening cash/bank. Items: product list with opening stock. Parties: customers &amp; suppliers with state and credit limit.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="127" t="inlineStr">
+      <c r="B6" s="133" t="inlineStr">
         <is>
           <t>2. Buy (Purchases)</t>
         </is>
       </c>
-      <c r="C6" s="128" t="inlineStr">
+      <c r="C6" s="134" t="inlineStr">
         <is>
           <t>Pick supplier and item from dropdowns, type qty. Rate blank = standard purchase rate. 'Paid Via' blank = on credit (creates payable).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="127" t="inlineStr">
+      <c r="B7" s="133" t="inlineStr">
         <is>
           <t>3. Stock updates itself</t>
         </is>
       </c>
-      <c r="C7" s="128" t="inlineStr">
+      <c r="C7" s="134" t="inlineStr">
         <is>
           <t>Items sheet instantly shows closing stock, weighted-average cost, stock value and REORDER / OUT OF STOCK / DEAD STOCK alerts.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="B8" s="127" t="inlineStr">
+      <c r="B8" s="133" t="inlineStr">
         <is>
           <t>4. Sell (Sales)</t>
         </is>
       </c>
-      <c r="C8" s="128" t="inlineStr">
+      <c r="C8" s="134" t="inlineStr">
         <is>
           <t>One line per item; keep all lines of an invoice together. CGST+SGST or IGST is chosen automatically from customer state vs. your home state. 'Stock Check' warns on negative stock or selling below cost.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="127" t="inlineStr">
+      <c r="B9" s="133" t="inlineStr">
         <is>
           <t>5. Print invoice</t>
         </is>
       </c>
-      <c r="C9" s="128" t="inlineStr">
+      <c r="C9" s="134" t="inlineStr">
         <is>
           <t>Invoice sheet shows the latest invoice automatically. Type any invoice number in the cream cell to reprint. Ctrl+P (fits one A4 page). Doubles as delivery challan.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="127" t="inlineStr">
+      <c r="B10" s="133" t="inlineStr">
         <is>
           <t>6. Deliver</t>
         </is>
       </c>
-      <c r="C10" s="128" t="inlineStr">
+      <c r="C10" s="134" t="inlineStr">
         <is>
           <t>Set the Delivery column (Pending / Packed / Dispatched / Delivered). Dashboard counts what is still pending.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="127" t="inlineStr">
+      <c r="B11" s="133" t="inlineStr">
         <is>
           <t>7. Collect &amp; pay (CashBook)</t>
         </is>
       </c>
-      <c r="C11" s="128" t="inlineStr">
+      <c r="C11" s="134" t="inlineStr">
         <is>
           <t>Receipt = money from customer; Payment = money to supplier; Expense = shop costs; Transfer In/Out moves money between Cash/Bank/UPI (enter both legs).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="127" t="inlineStr">
+      <c r="B12" s="133" t="inlineStr">
         <is>
           <t>8. Review</t>
         </is>
       </c>
-      <c r="C12" s="128" t="inlineStr">
+      <c r="C12" s="134" t="inlineStr">
         <is>
           <t>Dashboard for the live picture, Reports for monthly P&amp;L, GST rate-wise summary and expense analysis.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="126" t="inlineStr">
+      <c r="B14" s="132" t="inlineStr">
         <is>
           <t>PAIN POINTS THIS SOLVES</t>
         </is>
@@ -3907,103 +4055,103 @@
       <c r="C14" s="57" t="n"/>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="B15" s="127" t="inlineStr">
+      <c r="B15" s="133" t="inlineStr">
         <is>
           <t>Stock never matches</t>
         </is>
       </c>
-      <c r="C15" s="128" t="inlineStr">
+      <c r="C15" s="134" t="inlineStr">
         <is>
           <t>Single source of truth: stock = opening + purchases − sales ± adjustments. No manual stock register.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="B16" s="127" t="inlineStr">
+      <c r="B16" s="133" t="inlineStr">
         <is>
           <t>Don't know real profit</t>
         </is>
       </c>
-      <c r="C16" s="128" t="inlineStr">
+      <c r="C16" s="134" t="inlineStr">
         <is>
           <t>Every sale line carries COGS at weighted-average cost, so gross and net profit are exact per line, item, month.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="B17" s="127" t="inlineStr">
+      <c r="B17" s="133" t="inlineStr">
         <is>
           <t>Money stuck with customers</t>
         </is>
       </c>
-      <c r="C17" s="128" t="inlineStr">
+      <c r="C17" s="134" t="inlineStr">
         <is>
           <t>Party ledger with credit limit, credit days, OVERDUE / OVER LIMIT flags and Days Unpaid.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="B18" s="127" t="inlineStr">
+      <c r="B18" s="133" t="inlineStr">
         <is>
           <t>Running out / overstock</t>
         </is>
       </c>
-      <c r="C18" s="128" t="inlineStr">
+      <c r="C18" s="134" t="inlineStr">
         <is>
           <t>Reorder level + suggested order qty, days-of-cover, and dead-stock detection (no sale in N days).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="B19" s="127" t="inlineStr">
+      <c r="B19" s="133" t="inlineStr">
         <is>
           <t>GST headache</t>
         </is>
       </c>
-      <c r="C19" s="128" t="inlineStr">
+      <c r="C19" s="134" t="inlineStr">
         <is>
           <t>Automatic CGST/SGST vs IGST split, rate-wise output vs input summary per FY, net payable on dashboard.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="B20" s="127" t="inlineStr">
+      <c r="B20" s="133" t="inlineStr">
         <is>
           <t>Double entry for cash sales</t>
         </is>
       </c>
-      <c r="C20" s="128" t="inlineStr">
+      <c r="C20" s="134" t="inlineStr">
         <is>
           <t>'Paid Via' on the bill itself books cash/bank/UPI immediately - no separate receipt needed.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="B21" s="127" t="inlineStr">
+      <c r="B21" s="133" t="inlineStr">
         <is>
           <t>Typing errors</t>
         </is>
       </c>
-      <c r="C21" s="128" t="inlineStr">
+      <c r="C21" s="134" t="inlineStr">
         <is>
           <t>Dropdowns everywhere, unique-name checks, qty/date validation, row-level 'Check' columns.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="B22" s="127" t="inlineStr">
+      <c r="B22" s="133" t="inlineStr">
         <is>
           <t>Slow, crashing Excel files</t>
         </is>
       </c>
-      <c r="C22" s="128" t="inlineStr">
+      <c r="C22" s="134" t="inlineStr">
         <is>
           <t>See SPEED DESIGN below.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="126" t="inlineStr">
+      <c r="B24" s="132" t="inlineStr">
         <is>
           <t>SPEED DESIGN (why it stays fast)</t>
         </is>
@@ -4011,67 +4159,67 @@
       <c r="C24" s="57" t="n"/>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="B25" s="127" t="inlineStr">
+      <c r="B25" s="133" t="inlineStr">
         <is>
           <t>No volatile functions</t>
         </is>
       </c>
-      <c r="C25" s="128" t="inlineStr">
+      <c r="C25" s="134" t="inlineStr">
         <is>
           <t>No OFFSET/INDIRECT in cell formulas; TODAY() appears once (Settings!B10). Volatile names are used only by dropdowns, which are not recalculated.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="B26" s="127" t="inlineStr">
+      <c r="B26" s="133" t="inlineStr">
         <is>
           <t>Bounded ranges</t>
         </is>
       </c>
-      <c r="C26" s="128" t="inlineStr">
+      <c r="C26" s="134" t="inlineStr">
         <is>
           <t>All lookups use fixed ranges (20,000 transaction rows, 2000 items, 1000 parties) - never whole-column A:A references.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="B27" s="127" t="inlineStr">
+      <c r="B27" s="133" t="inlineStr">
         <is>
           <t>Match once, reuse</t>
         </is>
       </c>
-      <c r="C27" s="128" t="inlineStr">
+      <c r="C27" s="134" t="inlineStr">
         <is>
           <t>Each transaction row runs one MATCH into a hidden helper column, then several cheap INDEX calls reuse it.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="B28" s="127" t="inlineStr">
+      <c r="B28" s="133" t="inlineStr">
         <is>
           <t>SUMIFS engine</t>
         </is>
       </c>
-      <c r="C28" s="128" t="inlineStr">
+      <c r="C28" s="134" t="inlineStr">
         <is>
           <t>All aggregation uses SUMIFS/COUNTIFS - Excel's fastest multi-threaded aggregation functions. No SUMPRODUCT or array formulas.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
-      <c r="B29" s="127" t="inlineStr">
+      <c r="B29" s="133" t="inlineStr">
         <is>
           <t>Extra boost (optional)</t>
         </is>
       </c>
-      <c r="C29" s="128" t="inlineStr">
+      <c r="C29" s="134" t="inlineStr">
         <is>
           <t>Import ERP_Macros.bas (File &gt; Save As .xlsm, Alt+F11 &gt; File &gt; Import) for one-click Fast Mode, new invoice, PDF invoice, backup and archive.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="126" t="inlineStr">
+      <c r="B31" s="132" t="inlineStr">
         <is>
           <t>RULES &amp; LIMITS</t>
         </is>
@@ -4079,79 +4227,79 @@
       <c r="C31" s="57" t="n"/>
     </row>
     <row r="32" ht="28" customHeight="1">
-      <c r="B32" s="127" t="inlineStr">
+      <c r="B32" s="133" t="inlineStr">
         <is>
           <t>Colour code</t>
         </is>
       </c>
-      <c r="C32" s="128" t="inlineStr">
+      <c r="C32" s="134" t="inlineStr">
         <is>
           <t>Blue text on cream = you type. Black/grey = formula, never overwrite. Green = linked from another sheet.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
-      <c r="B33" s="127" t="inlineStr">
+      <c r="B33" s="133" t="inlineStr">
         <is>
           <t>Sample data</t>
         </is>
       </c>
-      <c r="C33" s="128" t="inlineStr">
+      <c r="C33" s="134" t="inlineStr">
         <is>
           <t>Rows already filled are DEMO data. Clear only the cream input cells (or run ClearDemoData macro) before going live.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
-      <c r="B34" s="127" t="inlineStr">
+      <c r="B34" s="133" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
       </c>
-      <c r="C34" s="128" t="inlineStr">
+      <c r="C34" s="134" t="inlineStr">
         <is>
           <t>20,000 lines per register per year. At year end: Save As a new file, set new FY start, carry forward closing stock as Opening Qty/Rate and party balances as Opening Bal.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
-      <c r="B35" s="127" t="inlineStr">
+      <c r="B35" s="133" t="inlineStr">
         <is>
           <t>Returns</t>
         </is>
       </c>
-      <c r="C35" s="128" t="inlineStr">
+      <c r="C35" s="134" t="inlineStr">
         <is>
           <t>Sales return: Adjustments with +qty, reason 'Sales Return', plus a Payment / credit in CashBook. Purchase return: −qty and a Receipt from supplier.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="28" customHeight="1">
-      <c r="B36" s="127" t="inlineStr">
+      <c r="B36" s="133" t="inlineStr">
         <is>
           <t>Costing method</t>
         </is>
       </c>
-      <c r="C36" s="128" t="inlineStr">
+      <c r="C36" s="134" t="inlineStr">
         <is>
           <t>Weighted-average cost over the year (opening + all purchases). COGS uses the current average, the standard method for traders.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1">
-      <c r="B37" s="127" t="inlineStr">
+      <c r="B37" s="133" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
       </c>
-      <c r="C37" s="128" t="inlineStr">
+      <c r="C37" s="134" t="inlineStr">
         <is>
           <t>Currency ₹ and Indian GST structure. Rates in Settings are editable; verify slabs with your CA.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="126" t="inlineStr">
+      <c r="B39" s="132" t="inlineStr">
         <is>
           <t>C ENGINE EDITION (SmartTrader64.xll)</t>
         </is>
@@ -4159,84 +4307,84 @@
       <c r="C39" s="57" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1">
-      <c r="B40" s="127" t="inlineStr">
+      <c r="B40" s="133" t="inlineStr">
         <is>
           <t>What it is</t>
         </is>
       </c>
-      <c r="C40" s="128" t="inlineStr">
+      <c r="C40" s="134" t="inlineStr">
         <is>
           <t>A native Excel add-in written in C. Stock, cost, GST, party ledgers and the cash book are posted in one pass by compiled code - six formulas instead of ~100,000. Results are identical to the formula edition, cell for cell.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
-      <c r="B41" s="127" t="inlineStr">
+      <c r="B41" s="133" t="inlineStr">
         <is>
           <t>Install once</t>
         </is>
       </c>
-      <c r="C41" s="128" t="inlineStr">
+      <c r="C41" s="134" t="inlineStr">
         <is>
           <t>1) Copy SmartTrader64.xll (or SmartTrader32.xll for 32-bit Office) to a folder, e.g. Documents\SmartTrader. 2) Right-click it &gt; Properties &gt; tick 'Unblock' &gt; OK (Windows blocks add-ins downloaded from the internet). 3) Excel &gt; File &gt; Options &gt; Add-ins &gt; Manage: Excel Add-ins &gt; Go &gt; Browse &gt; pick the .xll &gt; OK.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
-      <c r="B42" s="127" t="inlineStr">
+      <c r="B42" s="133" t="inlineStr">
         <is>
           <t>Check it works</t>
         </is>
       </c>
-      <c r="C42" s="128" t="inlineStr">
+      <c r="C42" s="134" t="inlineStr">
         <is>
           <t>Dashboard top-right shows 'Engine: SmartTrader C Engine 1.0'. A red '!! C engine not loaded' means step 3 was skipped and the grey columns show NAME errors until the add-in is loaded. Your typed data is never affected.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1">
-      <c r="B43" s="127" t="inlineStr">
+      <c r="B43" s="133" t="inlineStr">
         <is>
           <t>Which .xll?</t>
         </is>
       </c>
-      <c r="C43" s="128" t="inlineStr">
+      <c r="C43" s="134" t="inlineStr">
         <is>
           <t>Excel &gt; File &gt; Account &gt; About Excel shows '64-bit' or '32-bit'. Use the matching file.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
-      <c r="B44" s="127" t="inlineStr">
+      <c r="B44" s="133" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
       </c>
-      <c r="C44" s="128" t="inlineStr">
+      <c r="C44" s="134" t="inlineStr">
         <is>
           <t>20,000 lines per register, 2,000 items, 1,000 parties. A full recalculation of the sample data takes about 5 ms.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="28" customHeight="1">
-      <c r="B45" s="127" t="inlineStr">
+      <c r="B45" s="133" t="inlineStr">
         <is>
           <t>Do not</t>
         </is>
       </c>
-      <c r="C45" s="128" t="inlineStr">
+      <c r="C45" s="134" t="inlineStr">
         <is>
           <t>Sort the register sheets (the grey output blocks are single array formulas; use the filter arrows instead) or type inside grey columns.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="28" customHeight="1">
-      <c r="B46" s="127" t="inlineStr">
+      <c r="B46" s="133" t="inlineStr">
         <is>
           <t>Platforms</t>
         </is>
       </c>
-      <c r="C46" s="128" t="inlineStr">
+      <c r="C46" s="134" t="inlineStr">
         <is>
           <t>Excel for Windows (2010 and later, 32- or 64-bit). On Mac / Excel Online use the formula edition (SmartTrader_ERP.xlsx), which has the same layout.</t>
         </is>

</xml_diff>

<commit_message>
Rebuild workbooks and add-ins with the production licence secret
The secret is passed only through ST_LICENSE_KEYS at build time and never
appears in source. The harness licence tests now take their key from the
Makefile (made with the same secret), so they pass with any secret.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnFkPErZAiR8ShyLR6FSvf
</commit_message>
<xml_diff>
--- a/excel/SmartTrader_ERP_C.xlsx
+++ b/excel/SmartTrader_ERP_C.xlsx
@@ -4472,7 +4472,7 @@
     </row>
     <row r="6">
       <c r="A6">
-        <f>SUMPRODUCT(CODE(MID(A5,ROW($A$1:$A$40),1))*(MOD(ROW($A$1:$A$40)*7919,10007)+1))</f>
+        <f>SUMPRODUCT(CODE(MID(A5,ROW($A$1:$A$40),1))*(MOD(ROW($A$1:$A$40)*4517,9973)+1))</f>
         <v/>
       </c>
       <c r="B6" t="inlineStr">
@@ -4483,7 +4483,7 @@
     </row>
     <row r="7">
       <c r="A7">
-        <f>MOD(A6*9967+424242,1679616)</f>
+        <f>MOD(A6*8803+615290,1679616)</f>
         <v/>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>